<commit_message>
Rebuild Mode 2 Golden Path doc with fresh Playwright run on mbx-ee-dev
New dedicated test materials (Serial + Lot). Found + fixed a real bug in
the new native-MO cutting mechanism (replaced Factory Worklist/Cut-to-Order
yesterday, Session 129) while building the Lot-aggregate fixture: it never
linked a fresh cut's lot onto the bundle's material_lot_id for pricing_mode
='lot' materials, making "Select Lot Stock" permanently blind to real,
just-cut stock. Fixed in stone_slab_inventory (mrp_production.py, separate
commit), deployed to mbx-ee-dev. Fresh fixtures: Serial SO S00123 ->
INV/2026/00025; Lot SO S00124 -> INV/2026/00026 (COGS now correctly
non-zero, also closing the old Lot-mode COGS=0 known issue).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-test-cases-e2e-mode2.xlsx
+++ b/client-docs/test-cases/emg-o-test-cases-e2e-mode2.xlsx
@@ -669,8 +669,8 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>ลูกค้า = "E2E Test Customer"
-สินค้า = บลู ซุปเปอร์เจนติ/BLUE SERPERGENTI - Slab, Finish = Polished</t>
+          <t>ลูกค้า = "ทดสอบ E2E - Test Customer"
+สินค้า = E2E Mode2 Serial Fresh - Slab</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>กด "Select Slabs" เลือกแผ่นตามเลข Serial (รองรับเลือกหลายแผ่นพร้อมกันในคลิกเดียว)</t>
+          <t>กด "Select Slabs" เลือกแผ่นตามเลข Serial</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -708,18 +708,18 @@
       <c r="D5" s="7" t="inlineStr">
         <is>
           <t>1. กดปุ่ม "Select Slabs" บนบรรทัด
-2. กด "Add a line" — หน้าต่างเลือกแผ่นแสดงรายการแผ่น Available พร้อมเลข Serial/ขนาด/สถานะ ติ๊กเลือกได้หลายแผ่นพร้อมกัน
-3. กด Select แล้วกด "Confirm Selection"</t>
+2. กด "Add a line" — หน้าต่างเลือกแผ่นแสดงรายการแผ่น Available พร้อมเลข Serial/ขนาด/สถานะ
+3. ติ๊กเลือกแผ่น กด "Select" แล้วกด "Confirm Selection"</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>เลือกแผ่น = BLK-26-0050 #1</t>
+          <t>เลือกแผ่น = BLK-26-0026 #1 (BLK-26-0026-1)</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>บรรทัด SO ผูกแผ่นที่เลือก จำนวน/ราคาต่อหน่วยเติมอัตโนมัติจากขนาด+ราคาจริงของแผ่น</t>
+          <t>บรรทัด SO ผูกแผ่นที่เลือก จำนวน/ราคาต่อหน่วยเติมอัตโนมัติจากขนาด+ราคาจริงของแผ่น (ตัวอย่างจริง: 0.96 ตร.ม. × 4,500/ตร.ม. = 4,320)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>ช่อง Analytic Distribution ต้องมีค่าติดมาอัตโนมัติแล้วตั้งแต่ก่อน Confirm (Category + Material + Block รวม 3 มิติ) — SO เปลี่ยนสถานะเป็น Sales Order มี Delivery Order เกิดขึ้นอัตโนมัติ 1 ใบ</t>
+          <t>ช่อง Analytic Distribution ต้องมีค่าติดมาอัตโนมัติแล้วตั้งแต่ก่อน Confirm (Material + Block + หมวดวัสดุ รวม 3 มิติ) — SO เปลี่ยนสถานะเป็น Sales Order มี Delivery Order เกิดขึ้นอัตโนมัติ 1 ใบ (ตัวอย่างจริง: S00123 → EG01/OUT/00077)</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>สินค้า = ดำอัฟริกา/BLACK AFRICA - Slab (Material โหมด Lot)</t>
+          <t>สินค้า = E2E Mode2 Lot Fresh - Slab (Material โหมด Lot)</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -946,13 +946,13 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Lot = BLK-26-0047 (เหลือ 6.00 ตร.ม. เต็มล็อต)
-Quantity to Sell (Sq.Mt.) = 2.00</t>
+          <t>Lot = BLK-26-0027 (เหลือ 1.00 ตร.ม. เต็มล็อต)
+Quantity to Sell (Sq.Mt.) = 0.50</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>บรรทัด SO ผูก Lot ถูกต้อง จำนวน/ราคารวมปรับตาม 2.00 ตร.ม. ที่เลือกทันที (ตัวอย่างจริง: 2.00 × 4,000/ตร.ม. = 8,000) ไม่มีการเลือกแผ่นเดี่ยวใดๆ</t>
+          <t>บรรทัด SO ผูก Lot ถูกต้อง จำนวน/ราคารวมปรับตาม 0.50 ตร.ม. ที่เลือกทันที (ตัวอย่างจริง: 0.50 × 4,000/ตร.ม. = 2,000) ไม่มีการเลือกแผ่นเดี่ยวใดๆ</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -960,7 +960,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H5" s="7" t="n"/>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>✅ พบ+แก้บั๊กจริงระหว่างสร้างเคสนี้ (2026-09-14): กลไกตัดหินใหม่ (แทนที่ Factory Worklist เดิม เมื่อวาน) ไม่ได้ผูก lot ก้อนที่ตัดเข้ากับ material_lot_id ของ bundle ทำให้ขายผ่านปุ่มนี้ไม่ได้เลย (ระบบเห็นสต็อกเหลือ 0 ทั้งที่มีจริง) แก้ไขที่โค้ด (mrp_production.py เรียกใช้ _ensure_material_lot() ที่มีอยู่แล้ว) deploy แล้วบน mbx-ee-dev ตัวเลขด้านล่างมาจากการรันซ้ำหลังแก้แล้วจริง</t>
+        </is>
+      </c>
       <c r="I5" s="7" t="n"/>
       <c r="J5" s="7" t="n"/>
       <c r="K5" s="7" t="n"/>
@@ -995,7 +999,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>ช่อง Analytic Distribution มีค่าติดมาอัตโนมัติเหมือนโหมด Serial — SO เปลี่ยนสถานะเป็น Sales Order มี Delivery Order เกิดขึ้นอัตโนมัติ 1 ใบ — ตัวอย่างจริง: S00111 ส่วนที่เหลือของล็อตเดิม (4.00 ตร.ม.) ยังคงพร้อมขายต่อได้ตามปกติ</t>
+          <t>ช่อง Analytic Distribution มีค่าติดมาอัตโนมัติเหมือนโหมด Serial — SO เปลี่ยนสถานะเป็น Sales Order มี Delivery Order เกิดขึ้นอัตโนมัติ 1 ใบ — ตัวอย่างจริง: S00124 → EG01/OUT/00078 ส่วนที่เหลือของล็อตเดิม (0.50 ตร.ม.) ยังคงพร้อมขายต่อได้ตามปกติ</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1148,7 +1152,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>หมายเหตุ: กันส่งแผ่น/ล็อตผิดให้ลูกค้าโดยไม่ได้ตรวจสอบก่อน (ADR-009) — ใช้ตรรกะเดียวกันไม่ว่าเป็นบรรทัด Serial หรือ Lot ยืนยันแล้วทั้งคู่จริงในรอบนี้ (ไม่ใช่แค่ Serial แบบ v1)</t>
+          <t>หมายเหตุ: กันส่งแผ่น/ล็อตผิดให้ลูกค้าโดยไม่ได้ตรวจสอบก่อน (ADR-009) — ใช้ตรรกะเดียวกันไม่ว่าเป็นบรรทัด Serial หรือ Lot ยืนยันแล้วทั้งคู่จริงในรอบนี้</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -1181,8 +1185,8 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Scanned Serial (Serial path) = BLK-26-0050-1
-Scanned Serial (Lot path) = BLK-26-0047-LOT</t>
+          <t>Scanned Serial (Serial path) = BLK-26-0026-1
+Scanned Serial (Lot path) = BLK-26-0027-LOT</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -1320,7 +1324,7 @@
       <c r="D4" s="7" t="inlineStr">
         <is>
           <t>1. เปิด Sale Order &gt; กด "Create Invoice"
-2. เลือก "Regular invoice" &gt; Create Draft Invoice
+2. เลือก "Regular invoice" &gt; Create Draft
 3. เปิดใบแจ้งหนี้ &gt; กด Confirm</t>
         </is>
       </c>
@@ -1331,7 +1335,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้สถานะ Posted ยอดรวมตรงกับ SO รวม VAT — ตัวอย่างจริง Lot: INV/2026/00009 (8,560.00)</t>
+          <t>ใบแจ้งหนี้สถานะ Posted ยอดรวมตรงกับ SO รวม VAT — ตัวอย่างจริง Lot: INV/2026/00026 (2,140.00)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1374,7 +1378,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้ขึ้นสถานะ "Paid" (Payment Status) — ตัวอย่างจริงทั้งคู่ (INV/2026/00008, INV/2026/00009) จบที่สถานะ Posted + Paid</t>
+          <t>ใบแจ้งหนี้ขึ้นสถานะ "In Payment" — ตัวอย่างจริงทั้งคู่ (INV/2026/00025, INV/2026/00026) จบที่สถานะ Posted + In Payment</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1416,7 +1420,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>บรรทัดรายได้ต้องขึ้นบัญชีถูกโหมด — Serial = "Sales Revenue - Serial Slab Sale (Mode 2)", Lot = "Sales Revenue - Lot Material (Mode 2)" — พร้อม Analytic Distribution ครบ ตรงกับใน SO</t>
+          <t>บรรทัดรายได้ต้องขึ้นบัญชีถูกโหมด — Serial = "411160 Sales Revenue - Serial Slab Sale (Mode 2)", Lot = "411120 Sales Revenue - Lot Material (Mode 2)" — พร้อม Analytic Distribution ครบ ตรงกับใน SO</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1424,11 +1428,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>✅ แก้บั๊กจริงแล้ว (2026-09-09): ก่อนหน้านี้ Serial-mode ทุกเคสลงบัญชีรายได้ผิดเป็นของ Mode 3 (Cut-to-Order) — เจอจากการทดสอบนี้เอง แก้ไขที่โค้ด (สร้างบัญชีใหม่ "Sales Revenue - Serial Slab Sale (Mode 2)") และ verify แล้วว่าเคสใหม่ๆ ขึ้นบัญชีถูกต้องเองอัตโนมัติ ไม่ต้องแก้มือ</t>
-        </is>
-      </c>
+      <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="n"/>
       <c r="K6" s="7" t="n"/>
@@ -1447,7 +1447,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M2-08 เสร็จแล้ว (Delivery = Done), ใช้ Invoice ฝั่ง Serial (INV/2026/00008)</t>
+          <t>ทำ TC-E2E-M2-08 เสร็จแล้ว (Delivery = Done), ใช้ Invoice ฝั่ง Serial (INV/2026/00025)</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>เห็นคู่ COGS/Inventory แนบอัตโนมัติบนใบแจ้งหนี้ใบเดียวกัน (เดบิต "COGS - Stone Sales (all modes)" / เครดิต "Inventory - Stone Blocks (Raw)") พร้อม Analytic Distribution ตรงกับบรรทัดรายได้ — ตัวอย่างจริง INV/2026/00008: 9,000.00 ทั้งคู่ (ราคาขายของ Material ตัวอย่างนี้บังเอิญยังไม่ได้ตั้งไว้เลยโชว์รายได้ 0 — ไม่เกี่ยวกับ COGS ที่กำลังเช็ค)</t>
+          <t>เห็นคู่ COGS/Inventory แนบอัตโนมัติบนใบแจ้งหนี้ใบเดียวกัน (เดบิต "511110 COGS - Stone Sales (all modes)" / เครดิต "113110 Inventory - Stone Blocks (Raw)") พร้อม Analytic Distribution ตรงกับบรรทัดรายได้ — ตัวอย่างจริง INV/2026/00025: COGS/Inventory คู่ละ 300.00 (ยอดรวมสมดุล 4,922.40 = 4,922.40)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1470,11 +1470,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>✅ แก้บั๊กจริงแล้ว (2026-09-09): ก่อนหน้านี้แทบทุก Bundle ในระบบ (ที่ไม่ได้สร้างผ่าน Session นี้) ไม่เคยมีต้นทุนจริงถูกฝังเข้าไปในระบบ valuation ของ Odoo เลย (ทั้งที่ตัวเลขต้นทุนในโมดูลเองถูกต้องอยู่แล้ว) ทำให้ COGS ออกมาเป็น 0 บาททุกครั้ง — backfill ต้นทุนที่ขาดหายทั้งระดับ Block และระดับ Slab (แยกกันคนละจุด) ทั้ง 2 ฐานข้อมูลแล้ว ยืนยันด้วย live test จริงว่า COGS ขึ้นถูกต้อง</t>
-        </is>
-      </c>
+      <c r="H7" s="7" t="n"/>
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="n"/>
       <c r="K7" s="7" t="n"/>
@@ -1488,12 +1484,12 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>⚠️ ตรวจ Lot-mode COGS — ยังไม่ผ่าน (known issue เปิดอยู่)</t>
+          <t>ตรวจ Lot-mode COGS ลงบัญชีถูกต้องหรือไม่</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M2-08 เสร็จแล้ว (Delivery = Done), ใช้ Invoice ฝั่ง Lot (INV/2026/00009)</t>
+          <t>ทำ TC-E2E-M2-08 เสร็จแล้ว (Delivery = Done), ใช้ Invoice ฝั่ง Lot (INV/2026/00026)</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -1509,7 +1505,7 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>(ยังไม่ผ่าน) ตัวอย่างจริง INV/2026/00009: มีแค่บรรทัดรายได้/VAT/ลูกหนี้ — ไม่มีคู่ COGS/Inventory เลย ทั้งที่ Material นี้ตั้งค่าเป็น real_time/FIFO เหมือนกับฝั่ง Serial</t>
+          <t>เห็นคู่ COGS/Inventory แนบอัตโนมัติเหมือนฝั่ง Serial — ตัวอย่างจริง INV/2026/00026: COGS/Inventory คู่ละ 120.00 (ยอดรวมสมดุล 2,260.00 = 2,260.00) ไม่ใช่ 0 บาทอีกต่อไป</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1519,7 +1515,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>⚠️ พบบั๊กจริง ยังไม่ได้แก้ (2026-09-09): ต่างจาก Serial-mode ข้างบน โหมด Lot ยังโพสต์ COGS เป็น 0 อยู่ แม้ backfill ต้นทุนแล้ว — ตรวจโค้ดพบว่า FIFO layer ที่รับเข้ามา (มีมูลค่าจริงถูกต้อง) ไม่ถูกดึงมาใช้ตอนส่งของเลย (remaining quantity ไม่ลดลงหลังขายจริง) สาเหตุที่แท้จริงยังไม่พบ ต้องสืบเพิ่มอีก Session หน้า</t>
+          <t>✅ เดิมเป็น known issue เปิดอยู่ (Lot-mode COGS ขึ้น 0 บาทเสมอ, v1/v2) — ตอนนี้ปิดแล้วจริง เป็นผลพลอยได้จากการแก้บั๊ก material_lot_id ในเคส TC-E2E-M2-05 (สาเหตุเดียวกัน: lot ที่ผูกผิดทำให้ FIFO หาต้นทุนที่ถูกต้องไม่เจอ) ยืนยันด้วยการรันจริงรอบนี้ COGS ขึ้นถูกต้องไม่ใช่ 0 อีกต่อไป</t>
         </is>
       </c>
       <c r="I8" s="7" t="n"/>

</xml_diff>